<commit_message>
Modified get_active_jobs and test_run.py
</commit_message>
<xml_diff>
--- a/tests/fixtures/test_operations.xlsx
+++ b/tests/fixtures/test_operations.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cc3ab4ac00b3f12d/Desktop/essenn-production-vs-plan/tests/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cc3ab4ac00b3f12d/Desktop/essenn-production-vs-plan/tests/fixtures/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="4" documentId="11_F25DC773A252ABDACC1048C8E9DA48FA5BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E4B79218-4FE5-4212-9EFB-53AAA5D88821}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet13" sheetId="2" r:id="rId1"/>
@@ -506,11 +506,23 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="1"/>
@@ -522,18 +534,6 @@
       <alignment vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -552,10 +552,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -840,23 +836,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="14.1" customHeight="1">
-      <c r="A1" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
+      <c r="A1" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
-      <c r="J1" s="9" t="s">
+      <c r="J1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="K1" s="8"/>
-      <c r="L1" s="8"/>
-      <c r="M1" s="8"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
     </row>
     <row r="2" spans="1:13" ht="14.1" customHeight="1">
       <c r="A2" s="1"/>
@@ -874,21 +870,21 @@
       <c r="M2" s="1"/>
     </row>
     <row r="3" spans="1:13" ht="18" customHeight="1">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
-      <c r="K3" s="8"/>
-      <c r="L3" s="8"/>
-      <c r="M3" s="8"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="10"/>
+      <c r="L3" s="10"/>
+      <c r="M3" s="10"/>
     </row>
     <row r="4" spans="1:13" ht="15" customHeight="1">
       <c r="A4" s="1"/>
@@ -915,10 +911,10 @@
       <c r="C5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="12"/>
+      <c r="E5" s="16"/>
       <c r="F5" s="3" t="s">
         <v>7</v>
       </c>
@@ -928,10 +924,10 @@
       <c r="H5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I5" s="11" t="s">
+      <c r="I5" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="J5" s="12"/>
+      <c r="J5" s="16"/>
       <c r="K5" s="3" t="s">
         <v>11</v>
       </c>
@@ -950,10 +946,10 @@
       <c r="C6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="13">
+      <c r="D6" s="9">
         <v>315</v>
       </c>
-      <c r="E6" s="8"/>
+      <c r="E6" s="10"/>
       <c r="F6" s="4">
         <v>20</v>
       </c>
@@ -963,10 +959,10 @@
       <c r="H6" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I6" s="13" t="s">
+      <c r="I6" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="J6" s="8"/>
+      <c r="J6" s="10"/>
       <c r="K6" s="4" t="s">
         <v>19</v>
       </c>
@@ -985,10 +981,10 @@
       <c r="C7" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="14">
+      <c r="D7" s="11">
         <v>5867</v>
       </c>
-      <c r="E7" s="8"/>
+      <c r="E7" s="10"/>
       <c r="F7" s="5">
         <v>20</v>
       </c>
@@ -998,10 +994,10 @@
       <c r="H7" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I7" s="14" t="s">
+      <c r="I7" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="J7" s="8"/>
+      <c r="J7" s="10"/>
       <c r="K7" s="5" t="s">
         <v>25</v>
       </c>
@@ -1020,10 +1016,10 @@
       <c r="C8" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="13">
+      <c r="D8" s="9">
         <v>180</v>
       </c>
-      <c r="E8" s="8"/>
+      <c r="E8" s="10"/>
       <c r="F8" s="4">
         <v>1</v>
       </c>
@@ -1033,10 +1029,10 @@
       <c r="H8" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="I8" s="13" t="s">
+      <c r="I8" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="J8" s="8"/>
+      <c r="J8" s="10"/>
       <c r="K8" s="4" t="s">
         <v>33</v>
       </c>
@@ -1055,10 +1051,10 @@
       <c r="C9" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="D9" s="14">
+      <c r="D9" s="11">
         <v>961</v>
       </c>
-      <c r="E9" s="8"/>
+      <c r="E9" s="10"/>
       <c r="F9" s="5">
         <v>20</v>
       </c>
@@ -1068,10 +1064,10 @@
       <c r="H9" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="I9" s="14" t="s">
+      <c r="I9" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="J9" s="8"/>
+      <c r="J9" s="10"/>
       <c r="K9" s="5" t="s">
         <v>40</v>
       </c>
@@ -1090,10 +1086,10 @@
       <c r="C10" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="D10" s="13">
+      <c r="D10" s="9">
         <v>1060</v>
       </c>
-      <c r="E10" s="8"/>
+      <c r="E10" s="10"/>
       <c r="F10" s="4">
         <v>10</v>
       </c>
@@ -1103,10 +1099,10 @@
       <c r="H10" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="I10" s="13" t="s">
+      <c r="I10" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="J10" s="8"/>
+      <c r="J10" s="10"/>
       <c r="K10" s="4" t="s">
         <v>47</v>
       </c>
@@ -1125,10 +1121,10 @@
       <c r="C11" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="D11" s="14">
+      <c r="D11" s="11">
         <v>415</v>
       </c>
-      <c r="E11" s="8"/>
+      <c r="E11" s="10"/>
       <c r="F11" s="5">
         <v>20</v>
       </c>
@@ -1138,10 +1134,10 @@
       <c r="H11" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="I11" s="14" t="s">
+      <c r="I11" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="J11" s="8"/>
+      <c r="J11" s="10"/>
       <c r="K11" s="5" t="s">
         <v>53</v>
       </c>
@@ -1160,10 +1156,10 @@
       <c r="C12" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="D12" s="13">
+      <c r="D12" s="9">
         <v>1060</v>
       </c>
-      <c r="E12" s="8"/>
+      <c r="E12" s="10"/>
       <c r="F12" s="4">
         <v>10</v>
       </c>
@@ -1173,10 +1169,10 @@
       <c r="H12" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="I12" s="13" t="s">
+      <c r="I12" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="J12" s="8"/>
+      <c r="J12" s="10"/>
       <c r="K12" s="4" t="s">
         <v>47</v>
       </c>
@@ -1195,10 +1191,10 @@
       <c r="C13" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="D13" s="14">
+      <c r="D13" s="11">
         <v>415</v>
       </c>
-      <c r="E13" s="8"/>
+      <c r="E13" s="10"/>
       <c r="F13" s="5">
         <v>10</v>
       </c>
@@ -1208,10 +1204,10 @@
       <c r="H13" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="I13" s="14" t="s">
+      <c r="I13" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="J13" s="8"/>
+      <c r="J13" s="10"/>
       <c r="K13" s="5" t="s">
         <v>47</v>
       </c>
@@ -1230,10 +1226,10 @@
       <c r="C14" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="D14" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="E14" s="16"/>
+      <c r="D14" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E14" s="8"/>
       <c r="F14" s="6" t="s">
         <v>0</v>
       </c>
@@ -1243,10 +1239,10 @@
       <c r="H14" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="I14" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="J14" s="16"/>
+      <c r="I14" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="J14" s="8"/>
       <c r="K14" s="6" t="s">
         <v>0</v>
       </c>
@@ -1258,19 +1254,6 @@
     <row r="15" spans="1:13" ht="0" hidden="1" customHeight="1"/>
   </sheetData>
   <mergeCells count="23">
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="J1:M1"/>
-    <mergeCell ref="A3:M3"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="I8:J8"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="I9:J9"/>
     <mergeCell ref="D13:E13"/>
     <mergeCell ref="I13:J13"/>
     <mergeCell ref="D14:E14"/>
@@ -1281,6 +1264,19 @@
     <mergeCell ref="I11:J11"/>
     <mergeCell ref="D12:E12"/>
     <mergeCell ref="I12:J12"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="J1:M1"/>
+    <mergeCell ref="A3:M3"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="I5:J5"/>
   </mergeCells>
   <pageMargins left="0.98425196850393704" right="0.98425196850393704" top="0.98425196850393704" bottom="1.2482795275590599" header="0.98425196850393704" footer="0.98425196850393704"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
@@ -1311,23 +1307,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="14.1" customHeight="1">
-      <c r="A1" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
+      <c r="A1" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
-      <c r="J1" s="9" t="s">
+      <c r="J1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="K1" s="8"/>
-      <c r="L1" s="8"/>
-      <c r="M1" s="8"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
     </row>
     <row r="2" spans="1:13" ht="14.1" customHeight="1">
       <c r="A2" s="1"/>
@@ -1345,21 +1341,21 @@
       <c r="M2" s="1"/>
     </row>
     <row r="3" spans="1:13" ht="18" customHeight="1">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
-      <c r="K3" s="8"/>
-      <c r="L3" s="8"/>
-      <c r="M3" s="8"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="10"/>
+      <c r="L3" s="10"/>
+      <c r="M3" s="10"/>
     </row>
     <row r="4" spans="1:13" ht="14.4" customHeight="1">
       <c r="A4" s="1"/>
@@ -1386,10 +1382,10 @@
       <c r="C5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="12"/>
+      <c r="E5" s="16"/>
       <c r="F5" s="3" t="s">
         <v>7</v>
       </c>
@@ -1399,10 +1395,10 @@
       <c r="H5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I5" s="11" t="s">
+      <c r="I5" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="J5" s="12"/>
+      <c r="J5" s="16"/>
       <c r="K5" s="3" t="s">
         <v>11</v>
       </c>
@@ -1421,10 +1417,10 @@
       <c r="C6" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="D6" s="13">
+      <c r="D6" s="9">
         <v>325</v>
       </c>
-      <c r="E6" s="8"/>
+      <c r="E6" s="10"/>
       <c r="F6" s="4">
         <v>10</v>
       </c>
@@ -1434,10 +1430,10 @@
       <c r="H6" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="I6" s="13" t="s">
+      <c r="I6" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="J6" s="8"/>
+      <c r="J6" s="10"/>
       <c r="K6" s="4" t="s">
         <v>112</v>
       </c>
@@ -1456,10 +1452,10 @@
       <c r="C7" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="D7" s="14">
+      <c r="D7" s="11">
         <v>1580</v>
       </c>
-      <c r="E7" s="8"/>
+      <c r="E7" s="10"/>
       <c r="F7" s="5">
         <v>20</v>
       </c>
@@ -1469,10 +1465,10 @@
       <c r="H7" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="I7" s="14" t="s">
+      <c r="I7" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="J7" s="8"/>
+      <c r="J7" s="10"/>
       <c r="K7" s="5" t="s">
         <v>106</v>
       </c>
@@ -1491,10 +1487,10 @@
       <c r="C8" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="D8" s="13">
+      <c r="D8" s="9">
         <v>1050</v>
       </c>
-      <c r="E8" s="8"/>
+      <c r="E8" s="10"/>
       <c r="F8" s="4">
         <v>10</v>
       </c>
@@ -1504,10 +1500,10 @@
       <c r="H8" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="I8" s="13" t="s">
+      <c r="I8" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="J8" s="8"/>
+      <c r="J8" s="10"/>
       <c r="K8" s="4" t="s">
         <v>100</v>
       </c>
@@ -1526,10 +1522,10 @@
       <c r="C9" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="D9" s="14">
+      <c r="D9" s="11">
         <v>3398</v>
       </c>
-      <c r="E9" s="8"/>
+      <c r="E9" s="10"/>
       <c r="F9" s="5">
         <v>10</v>
       </c>
@@ -1539,10 +1535,10 @@
       <c r="H9" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="I9" s="14" t="s">
+      <c r="I9" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="J9" s="8"/>
+      <c r="J9" s="10"/>
       <c r="K9" s="5" t="s">
         <v>47</v>
       </c>
@@ -1561,10 +1557,10 @@
       <c r="C10" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="D10" s="13">
+      <c r="D10" s="9">
         <v>530</v>
       </c>
-      <c r="E10" s="8"/>
+      <c r="E10" s="10"/>
       <c r="F10" s="4">
         <v>10</v>
       </c>
@@ -1574,10 +1570,10 @@
       <c r="H10" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="I10" s="13" t="s">
+      <c r="I10" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="J10" s="8"/>
+      <c r="J10" s="10"/>
       <c r="K10" s="4" t="s">
         <v>89</v>
       </c>
@@ -1596,10 +1592,10 @@
       <c r="C11" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="D11" s="14">
+      <c r="D11" s="11">
         <v>2000</v>
       </c>
-      <c r="E11" s="8"/>
+      <c r="E11" s="10"/>
       <c r="F11" s="5">
         <v>10</v>
       </c>
@@ -1609,10 +1605,10 @@
       <c r="H11" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="14" t="s">
+      <c r="I11" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="J11" s="8"/>
+      <c r="J11" s="10"/>
       <c r="K11" s="5" t="s">
         <v>82</v>
       </c>
@@ -1631,10 +1627,10 @@
       <c r="C12" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="D12" s="13">
+      <c r="D12" s="9">
         <v>5023</v>
       </c>
-      <c r="E12" s="8"/>
+      <c r="E12" s="10"/>
       <c r="F12" s="4">
         <v>10</v>
       </c>
@@ -1644,10 +1640,10 @@
       <c r="H12" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="I12" s="13" t="s">
+      <c r="I12" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="J12" s="8"/>
+      <c r="J12" s="10"/>
       <c r="K12" s="4" t="s">
         <v>77</v>
       </c>
@@ -1666,10 +1662,10 @@
       <c r="C13" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="D13" s="14">
+      <c r="D13" s="11">
         <v>1060</v>
       </c>
-      <c r="E13" s="8"/>
+      <c r="E13" s="10"/>
       <c r="F13" s="5">
         <v>30</v>
       </c>
@@ -1679,10 +1675,10 @@
       <c r="H13" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="I13" s="14" t="s">
+      <c r="I13" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="J13" s="8"/>
+      <c r="J13" s="10"/>
       <c r="K13" s="5" t="s">
         <v>69</v>
       </c>
@@ -1701,10 +1697,10 @@
       <c r="C14" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="D14" s="13">
+      <c r="D14" s="9">
         <v>3100</v>
       </c>
-      <c r="E14" s="8"/>
+      <c r="E14" s="10"/>
       <c r="F14" s="4">
         <v>10</v>
       </c>
@@ -1714,10 +1710,10 @@
       <c r="H14" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="I14" s="13" t="s">
+      <c r="I14" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="J14" s="8"/>
+      <c r="J14" s="10"/>
       <c r="K14" s="4" t="s">
         <v>63</v>
       </c>
@@ -1736,10 +1732,10 @@
       <c r="C15" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="D15" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="E15" s="16"/>
+      <c r="D15" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E15" s="8"/>
       <c r="F15" s="6" t="s">
         <v>0</v>
       </c>
@@ -1749,10 +1745,10 @@
       <c r="H15" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="I15" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="J15" s="16"/>
+      <c r="I15" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="J15" s="8"/>
       <c r="K15" s="6" t="s">
         <v>0</v>
       </c>
@@ -1779,6 +1775,23 @@
     <row r="17" s="2" customFormat="1" ht="0" hidden="1" customHeight="1"/>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="J1:M1"/>
+    <mergeCell ref="A3:M3"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="I10:J10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="I11:J11"/>
     <mergeCell ref="D15:E15"/>
     <mergeCell ref="I15:J15"/>
     <mergeCell ref="D12:E12"/>
@@ -1787,23 +1800,6 @@
     <mergeCell ref="I13:J13"/>
     <mergeCell ref="D14:E14"/>
     <mergeCell ref="I14:J14"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="I9:J9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="I10:J10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="I11:J11"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="I8:J8"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="J1:M1"/>
-    <mergeCell ref="A3:M3"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="I5:J5"/>
   </mergeCells>
   <pageMargins left="0.98425196850393704" right="0.98425196850393704" top="0.98425196850393704" bottom="1.2482795275590599" header="0.98425196850393704" footer="0.98425196850393704"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>